<commit_message>
Fix live-deploy issues found in dev copy: loader abort, test placement, board date
- Config: add 'Import' to Updated By dropdown so loadPilotData no longer throws
  on the imported pilot rows (strict validation was aborting after row 1)
- LoadData: wrap each setValue in try/catch so no single cell can abort the load
- Tests: place harness rows in the first blank row INSIDE the formula range
  (formulas fill to row 500, so getLastRow()-based placement wrote past them and
  broke the 4 formula-dependent assertions #2/#13/#14/#16)
- Setup board QUERY: add "format <due> 'yyyy-mm-dd'" so Due shows a date, not a serial
- build_workbook.py: sync Updated By list; reference rebuilt; validate_logic ALL PASS
- Code.combined.gs regenerated (syntax-checked, no dup functions)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EvwbfcRzW8iihij2CBkwV3
</commit_message>
<xml_diff>
--- a/build/Twin_Visit_Logger_DEV_reference.xlsx
+++ b/build/Twin_Visit_Logger_DEV_reference.xlsx
@@ -6573,8 +6573,8 @@
     <dataValidation sqref="AV2:AV1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Allowed: Not Ready,Ready for Handoff,Handed Off to JM,JM Confirmed" type="list">
       <formula1>"Not Ready,Ready for Handoff,Handed Off to JM,JM Confirmed"</formula1>
     </dataValidation>
-    <dataValidation sqref="BB2:BB1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Allowed: Jonathan,Kyle,Cherry,Juan,JM,Apps Script" type="list">
-      <formula1>"Jonathan,Kyle,Cherry,Juan,JM,Apps Script"</formula1>
+    <dataValidation sqref="BB2:BB1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Allowed: Jonathan,Kyle,Cherry,Juan,JM,Apps Script,Import" type="list">
+      <formula1>"Jonathan,Kyle,Cherry,Juan,JM,Apps Script,Import"</formula1>
     </dataValidation>
     <dataValidation sqref="BC2:BC1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick a value from the list." prompt="Allowed: Manual,Apps Script,Import,TEST" type="list">
       <formula1>"Manual,Apps Script,Import,TEST"</formula1>
@@ -7197,6 +7197,11 @@
           <t>Jose Herrera</t>
         </is>
       </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Documents</t>

</xml_diff>